<commit_message>
Added the importer script to import COA and modified the COA Excel files
</commit_message>
<xml_diff>
--- a/Support Files/Accounts/Account Templates/Personales_2026.xlsx
+++ b/Support Files/Accounts/Account Templates/Personales_2026.xlsx
@@ -8,20 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lguevara/Documents/Desarrollos/MyAccountingBooks/Support Files/Accounts/Account Templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4B0568E-1BA9-1841-99A6-89C329B75B9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{520DDEA5-5CE9-7545-A9BD-22050FCBE532}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="100" yWindow="620" windowWidth="27860" windowHeight="15940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="COA" sheetId="1" r:id="rId1"/>
-    <sheet name="Template Data" sheetId="2" r:id="rId2"/>
+    <sheet name="Nodes" sheetId="1" r:id="rId1"/>
+    <sheet name="Meta" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1238" uniqueCount="631">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1241" uniqueCount="634">
   <si>
     <t>Kind</t>
   </si>
@@ -1877,27 +1877,6 @@
     <t>500-10.001.03-000.000</t>
   </si>
   <si>
-    <t>template_code</t>
-  </si>
-  <si>
-    <t>template_name</t>
-  </si>
-  <si>
-    <t>template_description</t>
-  </si>
-  <si>
-    <t>template_country</t>
-  </si>
-  <si>
-    <t>template_locale</t>
-  </si>
-  <si>
-    <t>template_industry</t>
-  </si>
-  <si>
-    <t>template_version</t>
-  </si>
-  <si>
     <t>PERSONALES_2026</t>
   </si>
   <si>
@@ -1914,16 +1893,52 @@
   </si>
   <si>
     <t>Type</t>
+  </si>
+  <si>
+    <t>Key</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>code</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>description</t>
+  </si>
+  <si>
+    <t>country</t>
+  </si>
+  <si>
+    <t>locale</t>
+  </si>
+  <si>
+    <t>industry</t>
+  </si>
+  <si>
+    <t>version</t>
+  </si>
+  <si>
+    <t>SYSTEM</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -2003,16 +2018,11 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{DBDAB7A7-5B62-FE4A-84A1-1226F37C8C84}" name="Table2" displayName="Table2" ref="A1:G2" totalsRowShown="0">
-  <autoFilter ref="A1:G2" xr:uid="{DBDAB7A7-5B62-FE4A-84A1-1226F37C8C84}"/>
-  <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{D79C4775-8117-1948-8764-C7C02B72B6E9}" name="template_code"/>
-    <tableColumn id="2" xr3:uid="{D6570D62-BDCC-304D-B958-C02634B4F053}" name="template_name"/>
-    <tableColumn id="3" xr3:uid="{F4156FF8-89E9-6F4B-B468-369E28C27C95}" name="template_description"/>
-    <tableColumn id="4" xr3:uid="{103AEB04-0AD9-E348-B49A-B43C8737A927}" name="template_country"/>
-    <tableColumn id="5" xr3:uid="{B4E30108-EADA-3E44-9E44-DBDC1E67AFD9}" name="template_locale"/>
-    <tableColumn id="6" xr3:uid="{902F4C0E-B4DB-0749-8A09-A48A22270B00}" name="template_industry"/>
-    <tableColumn id="7" xr3:uid="{15E04988-153B-254C-B007-5AAA1ED76C13}" name="template_version"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7B90B750-EF45-5742-B0E0-CD18CFC1119B}" name="Table3" displayName="Table3" ref="A1:B8" totalsRowShown="0">
+  <autoFilter ref="A1:B8" xr:uid="{7B90B750-EF45-5742-B0E0-CD18CFC1119B}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{DE64688C-41BB-3D4B-B8D2-131318064416}" name="Key"/>
+    <tableColumn id="2" xr3:uid="{D9E21AE2-72AF-6C4B-A88A-99EAAAF8B0F3}" name="Value"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2339,7 +2349,7 @@
         <v>1</v>
       </c>
       <c r="G1" t="s">
-        <v>630</v>
+        <v>623</v>
       </c>
       <c r="H1" t="s">
         <v>2</v>
@@ -2360,6 +2370,9 @@
       </c>
       <c r="F2">
         <v>0</v>
+      </c>
+      <c r="G2" t="s">
+        <v>633</v>
       </c>
       <c r="H2">
         <v>1</v>
@@ -10282,11 +10295,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF738BC3-E182-084E-A3E0-AADC092ED0F6}">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
-    <col min="2" max="2" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="42.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19.83203125" customWidth="1"/>
     <col min="4" max="4" width="17.1640625" customWidth="1"/>
     <col min="5" max="5" width="15.6640625" customWidth="1"/>
@@ -10294,50 +10307,69 @@
     <col min="7" max="7" width="16.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>624</v>
+      </c>
+      <c r="B1" t="s">
+        <v>625</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>626</v>
+      </c>
+      <c r="B2" t="s">
         <v>618</v>
       </c>
-      <c r="B1" t="s">
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>627</v>
+      </c>
+      <c r="B3" t="s">
         <v>619</v>
       </c>
-      <c r="C1" t="s">
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>628</v>
+      </c>
+      <c r="B4" t="s">
         <v>620</v>
       </c>
-      <c r="D1" t="s">
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>629</v>
+      </c>
+      <c r="B5" t="s">
         <v>621</v>
       </c>
-      <c r="E1" t="s">
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>630</v>
+      </c>
+      <c r="B6" t="s">
         <v>622</v>
       </c>
-      <c r="F1" t="s">
-        <v>623</v>
-      </c>
-      <c r="G1" t="s">
-        <v>624</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>625</v>
-      </c>
-      <c r="B2" t="s">
-        <v>626</v>
-      </c>
-      <c r="C2" t="s">
-        <v>627</v>
-      </c>
-      <c r="D2" t="s">
-        <v>628</v>
-      </c>
-      <c r="E2" t="s">
-        <v>629</v>
-      </c>
-      <c r="G2">
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>631</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>632</v>
+      </c>
+      <c r="B8">
         <v>1</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>